<commit_message>
Milestone: Đồng bộ và dọn dẹp toàn bộ source code, xóa các file rác và file txt cũ
</commit_message>
<xml_diff>
--- a/carlist/topdownracing.xlsx
+++ b/carlist/topdownracing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2D Sideway Showdown\carlist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB15708D-EFE6-4A71-A8AC-74D57CA88ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B03E426-0E06-4A1E-B1EA-E4C2B3A4F62B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19230" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1072,7 +1072,7 @@
         <v>37</v>
       </c>
       <c r="H11" s="10">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="I11" s="13">
         <v>1.4</v>

</xml_diff>